<commit_message>
Added Launch/Stop to the Common.js
</commit_message>
<xml_diff>
--- a/FWInfragisticsOutlookCRM/TestCases/!Template/Main.rvl.xlsx
+++ b/FWInfragisticsOutlookCRM/TestCases/!Template/Main.rvl.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="23" uniqueCount="17">
   <si>
     <t>Flow</t>
   </si>
@@ -56,6 +56,15 @@
   </si>
   <si>
     <t>Shared\OutlookCRM.exe.lnk</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Application is started in Common.js</t>
+  </si>
+  <si>
+    <t>Application is always started in Common.js</t>
   </si>
 </sst>
 </file>
@@ -76,7 +85,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -85,13 +94,15 @@
       <diagonal/>
     </border>
     <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -101,7 +112,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.34375" customWidth="true"/>
@@ -151,25 +162,17 @@
       <c r="H2" s="1"/>
     </row>
     <row r="3">
-      <c r="A3" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>12</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
       <c r="H3" s="1"/>
     </row>
     <row r="4">
@@ -332,16 +335,7 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
     </row>
-    <row r="20">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-    </row>
   </sheetData>
+  <tableParts/>
 </worksheet>
 </file>
</xml_diff>